<commit_message>
Change Acquisition Function from qnehvi to qehvi, since no noise is required and pruning is expensive.
</commit_message>
<xml_diff>
--- a/batch_pareto_0407_cpugpu_checkpoint.xlsx
+++ b/batch_pareto_0407_cpugpu_checkpoint.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,574 +461,574 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.4605907698598534</v>
+        <v>0.6241361421975099</v>
       </c>
       <c r="B2" t="n">
-        <v>0.00536663395895672</v>
+        <v>0.01436610877026545</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05605854974409318</v>
+        <v>0.1092749338337411</v>
       </c>
       <c r="D2" t="n">
-        <v>0.05488037881227441</v>
+        <v>0.01836842916982555</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4605907698598535</v>
+        <v>0.6241361421975097</v>
       </c>
       <c r="F2" t="n">
-        <v>25.39580109128971</v>
+        <v>23.61702076828051</v>
       </c>
       <c r="G2" t="n">
-        <v>71.07490914010883</v>
+        <v>74.52703529819331</v>
       </c>
       <c r="H2" t="n">
-        <v>4286.953261662765</v>
+        <v>2170.079650746617</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.4607728448652993</v>
+        <v>0.6549829378958806</v>
       </c>
       <c r="B3" t="n">
-        <v>0.02056303118017329</v>
+        <v>0.04571167652724498</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1968776615030081</v>
+        <v>0.07292338050001514</v>
       </c>
       <c r="D3" t="n">
-        <v>0.07066220218593261</v>
+        <v>0.1889329842573734</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4607728448652997</v>
+        <v>0.6549829378958811</v>
       </c>
       <c r="F3" t="n">
-        <v>77.68890333046036</v>
+        <v>49.18051262777236</v>
       </c>
       <c r="G3" t="n">
-        <v>27.27528370100381</v>
+        <v>46.52659880333209</v>
       </c>
       <c r="H3" t="n">
-        <v>1119.270957640387</v>
+        <v>715.7120506923368</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.7265117402976299</v>
+        <v>0.5081052830004644</v>
       </c>
       <c r="B4" t="n">
-        <v>0.01532666502756333</v>
+        <v>0.0340489651914698</v>
       </c>
       <c r="C4" t="n">
-        <v>0.07788943396765398</v>
+        <v>0.1166620745657937</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1012382157346449</v>
+        <v>0.1618816358663217</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7265117402976309</v>
+        <v>0.5081052830004649</v>
       </c>
       <c r="F4" t="n">
-        <v>44.57875990411124</v>
+        <v>72.98711469056548</v>
       </c>
       <c r="G4" t="n">
-        <v>71.19509287394041</v>
+        <v>32.20619757561012</v>
       </c>
       <c r="H4" t="n">
-        <v>2367.720659556683</v>
+        <v>745.3929581458042</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.5141074403162238</v>
+        <v>0.3652628068453664</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0006009361489155125</v>
+        <v>0.01246855704094606</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1469494691530456</v>
+        <v>0.1362367332246552</v>
       </c>
       <c r="D5" t="n">
-        <v>0.08721747057920672</v>
+        <v>0.1415669667998128</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5141074403162241</v>
+        <v>0.3652628068453668</v>
       </c>
       <c r="F5" t="n">
-        <v>15.99021582907613</v>
+        <v>74.87098588429849</v>
       </c>
       <c r="G5" t="n">
-        <v>36.03797396783027</v>
+        <v>22.62723250719103</v>
       </c>
       <c r="H5" t="n">
-        <v>42732.77067811371</v>
+        <v>1463.270941618256</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.6821222462345157</v>
+        <v>0.5724057673080921</v>
       </c>
       <c r="B6" t="n">
-        <v>0.001950634506101156</v>
+        <v>0.01965918048850201</v>
       </c>
       <c r="C6" t="n">
-        <v>0.115852760964206</v>
+        <v>0.1151436126657707</v>
       </c>
       <c r="D6" t="n">
-        <v>0.117259099084879</v>
+        <v>0.1963646205330634</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6821222462345168</v>
+        <v>0.5724057673080927</v>
       </c>
       <c r="F6" t="n">
-        <v>35.69513989660046</v>
+        <v>71.62095974698143</v>
       </c>
       <c r="G6" t="n">
-        <v>50.24058087855256</v>
+        <v>33.03097639383443</v>
       </c>
       <c r="H6" t="n">
-        <v>17467.14009869317</v>
+        <v>1454.367240473806</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.540073891707468</v>
+        <v>0.4100526373163189</v>
       </c>
       <c r="B7" t="n">
-        <v>0.03640581758124277</v>
+        <v>0.006008430930982275</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1895483414661987</v>
+        <v>0.1585017101569662</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1756536892642499</v>
+        <v>0.02141475488284207</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5400738917074684</v>
+        <v>0.4100526373163195</v>
       </c>
       <c r="F7" t="n">
-        <v>109.8954265438962</v>
+        <v>26.08810965552059</v>
       </c>
       <c r="G7" t="n">
-        <v>25.19524633888532</v>
+        <v>34.46961185358417</v>
       </c>
       <c r="H7" t="n">
-        <v>740.9994523701391</v>
+        <v>3408.898174785484</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.6401734934202166</v>
+        <v>0.5339045460632239</v>
       </c>
       <c r="B8" t="n">
-        <v>0.03910531173058714</v>
+        <v>0.03243572651478052</v>
       </c>
       <c r="C8" t="n">
-        <v>0.05911096540644827</v>
+        <v>0.1882809194674129</v>
       </c>
       <c r="D8" t="n">
-        <v>0.008662321283442433</v>
+        <v>0.1730411358487552</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6401734934202167</v>
+        <v>0.5339045460632248</v>
       </c>
       <c r="F8" t="n">
-        <v>12.36571929020495</v>
+        <v>108.3606742830358</v>
       </c>
       <c r="G8" t="n">
-        <v>143.2492687569575</v>
+        <v>25.1567384594804</v>
       </c>
       <c r="H8" t="n">
-        <v>817.7064593332085</v>
+        <v>822.1962305578551</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.6143736751296418</v>
+        <v>0.4977970707578255</v>
       </c>
       <c r="B9" t="n">
-        <v>0.0237222657206872</v>
+        <v>0.04846411143502144</v>
       </c>
       <c r="C9" t="n">
-        <v>0.09733823025716073</v>
+        <v>0.1299525177063411</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1350173343354855</v>
+        <v>0.1086032502599535</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6143736751296426</v>
+        <v>0.4977970707578261</v>
       </c>
       <c r="F9" t="n">
-        <v>59.30334692059868</v>
+        <v>74.39595920268646</v>
       </c>
       <c r="G9" t="n">
-        <v>46.68145190489906</v>
+        <v>35.23498220686869</v>
       </c>
       <c r="H9" t="n">
-        <v>1293.635499831867</v>
+        <v>513.0593123055868</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.5795068285313367</v>
+        <v>0.7683715717255378</v>
       </c>
       <c r="B10" t="n">
-        <v>0.0438238431228001</v>
+        <v>0.04322557262478177</v>
       </c>
       <c r="C10" t="n">
-        <v>0.1435516203079684</v>
+        <v>0.0822984428131502</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1267068992942932</v>
+        <v>0.03726240135157408</v>
       </c>
       <c r="E10" t="n">
-        <v>0.5795068285313373</v>
+        <v>0.768371571725539</v>
       </c>
       <c r="F10" t="n">
-        <v>82.51346278585206</v>
+        <v>35.62212765458479</v>
       </c>
       <c r="G10" t="n">
-        <v>36.37800671118937</v>
+        <v>103.3744631095427</v>
       </c>
       <c r="H10" t="n">
-        <v>660.5163769874958</v>
+        <v>887.9040271102571</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.7414385592098276</v>
+        <v>0.5187607875381867</v>
       </c>
       <c r="B11" t="n">
-        <v>0.006951034528663112</v>
+        <v>0.02799791629256348</v>
       </c>
       <c r="C11" t="n">
-        <v>0.1091763711349402</v>
+        <v>0.02507587145882896</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1035820419936312</v>
+        <v>0.004012817885387252</v>
       </c>
       <c r="E11" t="n">
-        <v>0.7414385592098279</v>
+        <v>0.5187607875381869</v>
       </c>
       <c r="F11" t="n">
-        <v>51.28717218201987</v>
+        <v>5.150408476496328</v>
       </c>
       <c r="G11" t="n">
-        <v>59.49491443993791</v>
+        <v>271.3114545312241</v>
       </c>
       <c r="H11" t="n">
-        <v>5327.963180130228</v>
+        <v>925.5010646779791</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.3925612911092625</v>
+        <v>0.5738978456114175</v>
       </c>
       <c r="B12" t="n">
-        <v>0.03697135417635599</v>
+        <v>0.02746355094454894</v>
       </c>
       <c r="C12" t="n">
-        <v>0.02736502620597219</v>
+        <v>0.1292640901970849</v>
       </c>
       <c r="D12" t="n">
-        <v>0.01923163686047533</v>
+        <v>0.08814754341215358</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3925612911092629</v>
+        <v>0.5738978456114183</v>
       </c>
       <c r="F12" t="n">
-        <v>14.60466994618967</v>
+        <v>67.12842029940482</v>
       </c>
       <c r="G12" t="n">
-        <v>140.188868453865</v>
+        <v>43.81613594198203</v>
       </c>
       <c r="H12" t="n">
-        <v>530.3683602546455</v>
+        <v>1043.790638951591</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.4221450596621921</v>
+        <v>0.5189204785244544</v>
       </c>
       <c r="B13" t="n">
-        <v>0.007502757497779529</v>
+        <v>0.02078481053814979</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1701876252006789</v>
+        <v>0.07036344509167938</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1466994798693478</v>
+        <v>0.02208000900886508</v>
       </c>
       <c r="E13" t="n">
-        <v>0.4221450596621927</v>
+        <v>0.518920478524455</v>
       </c>
       <c r="F13" t="n">
-        <v>82.74227359229201</v>
+        <v>25.08373357659623</v>
       </c>
       <c r="G13" t="n">
-        <v>22.55415503106996</v>
+        <v>88.17486889190366</v>
       </c>
       <c r="H13" t="n">
-        <v>2810.452788373744</v>
+        <v>1247.068278766418</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.4724030143093583</v>
+        <v>0.6393748789825016</v>
       </c>
       <c r="B14" t="n">
-        <v>0.03011493029289751</v>
+        <v>0.03196578607467276</v>
       </c>
       <c r="C14" t="n">
-        <v>0.1468626444228607</v>
+        <v>0.009652782085840686</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1494216089106953</v>
+        <v>0.04162982748027934</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4724030143093587</v>
+        <v>0.6393748789825024</v>
       </c>
       <c r="F14" t="n">
-        <v>86.41836279699008</v>
+        <v>5.964662157619421</v>
       </c>
       <c r="G14" t="n">
-        <v>27.38798594404518</v>
+        <v>240.1821367250768</v>
       </c>
       <c r="H14" t="n">
-        <v>783.5492340594118</v>
+        <v>999.0924399785119</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.5909512090610783</v>
+        <v>0.5942565913854085</v>
       </c>
       <c r="B15" t="n">
-        <v>0.001968818934140077</v>
+        <v>0.0225279139612987</v>
       </c>
       <c r="C15" t="n">
-        <v>0.1946960626449909</v>
+        <v>0.156279261920159</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1414299112641797</v>
+        <v>0.1878908098586485</v>
       </c>
       <c r="E15" t="n">
-        <v>0.5909512090610791</v>
+        <v>0.5942565913854094</v>
       </c>
       <c r="F15" t="n">
-        <v>56.33619985881422</v>
+        <v>92.85317199095327</v>
       </c>
       <c r="G15" t="n">
-        <v>29.33619717632636</v>
+        <v>30.10031560237066</v>
       </c>
       <c r="H15" t="n">
-        <v>14992.75143119929</v>
+        <v>1317.614972726488</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.601886791727917</v>
+        <v>0.6809831026531104</v>
       </c>
       <c r="B16" t="n">
-        <v>0.0240510494989531</v>
+        <v>0.02212414851393726</v>
       </c>
       <c r="C16" t="n">
-        <v>0.08154826553019907</v>
+        <v>0.09409129718625681</v>
       </c>
       <c r="D16" t="n">
-        <v>0.05878516489366851</v>
+        <v>0.06061767351319798</v>
       </c>
       <c r="E16" t="n">
-        <v>0.6018867917279179</v>
+        <v>0.6809831026531107</v>
       </c>
       <c r="F16" t="n">
-        <v>42.35033388592814</v>
+        <v>46.16653946167082</v>
       </c>
       <c r="G16" t="n">
-        <v>71.52046067352784</v>
+        <v>72.72657763783852</v>
       </c>
       <c r="H16" t="n">
-        <v>1250.018018885958</v>
+        <v>1537.465089609882</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.5999654838711365</v>
+        <v>0.2012227561737309</v>
       </c>
       <c r="B17" t="n">
-        <v>0.007121289879656969</v>
+        <v>0.003306733881589567</v>
       </c>
       <c r="C17" t="n">
-        <v>0.1899874694941245</v>
+        <v>0.1849030474049129</v>
       </c>
       <c r="D17" t="n">
-        <v>0.08481027532798542</v>
+        <v>0.1102092601526359</v>
       </c>
       <c r="E17" t="n">
-        <v>0.599965483871137</v>
+        <v>0.2012227561737312</v>
       </c>
       <c r="F17" t="n">
-        <v>69.26989221548092</v>
+        <v>63.16567646719312</v>
       </c>
       <c r="G17" t="n">
-        <v>35.08404761479756</v>
+        <v>11.19609646687538</v>
       </c>
       <c r="H17" t="n">
-        <v>4208.265135361522</v>
+        <v>3039.578336447883</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.6048109324558681</v>
+        <v>0.3452143917891028</v>
       </c>
       <c r="B18" t="n">
-        <v>0.03378751210377478</v>
+        <v>0.01234622474488356</v>
       </c>
       <c r="C18" t="n">
-        <v>0.1303273021856727</v>
+        <v>0.1803226609586051</v>
       </c>
       <c r="D18" t="n">
-        <v>0.08131138622543482</v>
+        <v>0.136104239428006</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6048109324558683</v>
+        <v>0.345214391789103</v>
       </c>
       <c r="F18" t="n">
-        <v>66.16621229532431</v>
+        <v>91.55047846704277</v>
       </c>
       <c r="G18" t="n">
-        <v>47.09523105596454</v>
+        <v>18.26265808770979</v>
       </c>
       <c r="H18" t="n">
-        <v>894.1263856120227</v>
+        <v>1396.658430101204</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.6124488142965134</v>
+        <v>0.7504553892184465</v>
       </c>
       <c r="B19" t="n">
-        <v>0.0206292065179416</v>
+        <v>0.02371617243641781</v>
       </c>
       <c r="C19" t="n">
-        <v>0.02090830977632728</v>
+        <v>0.1112044311572303</v>
       </c>
       <c r="D19" t="n">
-        <v>0.007544488837450056</v>
+        <v>0.02486282003860534</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6124488142965143</v>
+        <v>0.7504553892184468</v>
       </c>
       <c r="F19" t="n">
-        <v>7.06659370929658</v>
+        <v>30.41257982693442</v>
       </c>
       <c r="G19" t="n">
-        <v>341.0063127652275</v>
+        <v>85.09568454653161</v>
       </c>
       <c r="H19" t="n">
-        <v>1482.937225312305</v>
+        <v>1580.577422092793</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.6402142552925887</v>
+        <v>0.6391473829711666</v>
       </c>
       <c r="B20" t="n">
-        <v>0.02101318600724855</v>
+        <v>0.01351710645294358</v>
       </c>
       <c r="C20" t="n">
-        <v>0.1502689238400826</v>
+        <v>0.1225383381966697</v>
       </c>
       <c r="D20" t="n">
-        <v>0.055505186806743</v>
+        <v>0.138712489469482</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6402142552925896</v>
+        <v>0.6391473829711677</v>
       </c>
       <c r="F20" t="n">
-        <v>57.81667132348547</v>
+        <v>68.19338905092552</v>
       </c>
       <c r="G20" t="n">
-        <v>49.36272898577743</v>
+        <v>42.42236343548252</v>
       </c>
       <c r="H20" t="n">
-        <v>1521.839764842595</v>
+        <v>2361.852508193978</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.5858234165834131</v>
+        <v>0.8</v>
       </c>
       <c r="B21" t="n">
-        <v>0.02341504058788233</v>
+        <v>0.004566015927303234</v>
       </c>
       <c r="C21" t="n">
-        <v>0.1421600068405595</v>
+        <v>0.03023052552081541</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1113838329002432</v>
+        <v>0.04592153167212629</v>
       </c>
       <c r="E21" t="n">
-        <v>0.5858234165834134</v>
+        <v>0.8000000000000007</v>
       </c>
       <c r="F21" t="n">
-        <v>76.22605309483286</v>
+        <v>12.17760140293474</v>
       </c>
       <c r="G21" t="n">
-        <v>38.80013838073066</v>
+        <v>186.9555505248495</v>
       </c>
       <c r="H21" t="n">
-        <v>1249.704417488177</v>
+        <v>8751.612047836439</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.64305864041006</v>
+        <v>0.8</v>
       </c>
       <c r="B22" t="n">
-        <v>0.03259834946544112</v>
+        <v>0.001399351699724725</v>
       </c>
       <c r="C22" t="n">
-        <v>0.07231199961471331</v>
+        <v>0.05987184187288615</v>
       </c>
       <c r="D22" t="n">
-        <v>0.02789066905727226</v>
+        <v>0.084643568688178</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6430586404100602</v>
+        <v>0.8000000000000006</v>
       </c>
       <c r="F22" t="n">
-        <v>29.13305680863925</v>
+        <v>13.49349348879035</v>
       </c>
       <c r="G22" t="n">
-        <v>102.106579187605</v>
+        <v>97.8968665919982</v>
       </c>
       <c r="H22" t="n">
-        <v>985.3498601987529</v>
+        <v>28556.08065353461</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.7067452402440453</v>
+        <v>0.8</v>
       </c>
       <c r="B23" t="n">
-        <v>0.01573833151310371</v>
+        <v>0.004806141100477421</v>
       </c>
       <c r="C23" t="n">
-        <v>0.101381596283956</v>
+        <v>0.05636289792077395</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0787674662125985</v>
+        <v>0.05462294544181671</v>
       </c>
       <c r="E23" t="n">
-        <v>0.7067452402440456</v>
+        <v>0.8000000000000012</v>
       </c>
       <c r="F23" t="n">
-        <v>51.19540555710709</v>
+        <v>22.77103791468128</v>
       </c>
       <c r="G23" t="n">
-        <v>65.83251885250998</v>
+        <v>123.2883302675275</v>
       </c>
       <c r="H23" t="n">
-        <v>2243.053828215378</v>
+        <v>8314.362638256813</v>
       </c>
     </row>
     <row r="24">
@@ -1036,77 +1036,181 @@
         <v>0.8</v>
       </c>
       <c r="B24" t="n">
-        <v>0.004398661202011376</v>
+        <v>0.001084968636790078</v>
       </c>
       <c r="C24" t="n">
-        <v>0.06357524307243659</v>
+        <v>0.04728999035584666</v>
       </c>
       <c r="D24" t="n">
-        <v>0.03516896010798456</v>
+        <v>0.08769617580859053</v>
       </c>
       <c r="E24" t="n">
-        <v>0.8</v>
+        <v>0.8000000000000007</v>
       </c>
       <c r="F24" t="n">
-        <v>19.6017888797213</v>
+        <v>6.845126783335862</v>
       </c>
       <c r="G24" t="n">
-        <v>132.2616212350694</v>
+        <v>107.2974950508589</v>
       </c>
       <c r="H24" t="n">
-        <v>9084.58236831867</v>
+        <v>36830.55771844541</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.7415454656710939</v>
+        <v>0.4946347183230081</v>
       </c>
       <c r="B25" t="n">
-        <v>0.002337266209953689</v>
+        <v>0.001109913682521748</v>
       </c>
       <c r="C25" t="n">
-        <v>0.07972360100187588</v>
+        <v>0.09059853732407544</v>
       </c>
       <c r="D25" t="n">
-        <v>0.06806552053299858</v>
+        <v>0.072326874220563</v>
       </c>
       <c r="E25" t="n">
-        <v>0.7415454656710943</v>
+        <v>0.4946347183230085</v>
       </c>
       <c r="F25" t="n">
-        <v>23.72666835220684</v>
+        <v>18.15188755284447</v>
       </c>
       <c r="G25" t="n">
-        <v>84.88007832238472</v>
+        <v>51.06306143887457</v>
       </c>
       <c r="H25" t="n">
-        <v>15847.6581967978</v>
+        <v>22260.29336272294</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
+        <v>0.7636193199929181</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.03035729925128324</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.01306102671601468</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.00652100286799571</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.7636193199929184</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4.488888156939739</v>
+      </c>
+      <c r="G26" t="n">
+        <v>631.7137878559565</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1256.461739824695</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>0.09864657182688037</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0.0004999999999999999</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.1011334169637965</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.09864657182688052</v>
+      </c>
+      <c r="F27" t="n">
+        <v>18.37922933235357</v>
+      </c>
+      <c r="G27" t="n">
+        <v>5.311696433596246</v>
+      </c>
+      <c r="H27" t="n">
+        <v>9854.792525505354</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
         <v>0.8</v>
       </c>
-      <c r="B26" t="n">
-        <v>0.005012974051785014</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.02971835848749996</v>
-      </c>
-      <c r="D26" t="n">
-        <v>0.01733489491883598</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0.8000000000000006</v>
-      </c>
-      <c r="F26" t="n">
-        <v>7.691238750081617</v>
-      </c>
-      <c r="G26" t="n">
-        <v>278.7024380578271</v>
-      </c>
-      <c r="H26" t="n">
-        <v>7971.315946822244</v>
+      <c r="B28" t="n">
+        <v>0.007514497722407658</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.04312136758474128</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.04557282319201623</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.8000000000000004</v>
+      </c>
+      <c r="F28" t="n">
+        <v>19.91747107002969</v>
+      </c>
+      <c r="G28" t="n">
+        <v>155.455914891337</v>
+      </c>
+      <c r="H28" t="n">
+        <v>5317.720688216097</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>0.3440263925636659</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0.006101701284415531</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.07139084231251946</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.07034995462145296</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.3440263925636661</v>
+      </c>
+      <c r="F29" t="n">
+        <v>34.07161543979756</v>
+      </c>
+      <c r="G29" t="n">
+        <v>41.57496199296074</v>
+      </c>
+      <c r="H29" t="n">
+        <v>2816.28311639008</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>0.5606470561538109</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0.002127492979362342</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.04443107812176497</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.04217889203797519</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.5606470561538112</v>
+      </c>
+      <c r="F30" t="n">
+        <v>12.54453982250854</v>
+      </c>
+      <c r="G30" t="n">
+        <v>110.5185474974778</v>
+      </c>
+      <c r="H30" t="n">
+        <v>13163.06127754009</v>
       </c>
     </row>
   </sheetData>
@@ -1120,7 +1224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1145,10 +1249,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>70494669.7914847</v>
+        <v>30190010.59769762</v>
       </c>
       <c r="C2" t="n">
-        <v>19.45272709999699</v>
+        <v>17.27276129999518</v>
       </c>
     </row>
     <row r="3">
@@ -1156,10 +1260,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>70494669.7914847</v>
+        <v>30190010.59769762</v>
       </c>
       <c r="C3" t="n">
-        <v>15.70393169999443</v>
+        <v>15.41279600000416</v>
       </c>
     </row>
     <row r="4">
@@ -1167,10 +1271,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>80215041.95503481</v>
+        <v>30190010.59769762</v>
       </c>
       <c r="C4" t="n">
-        <v>14.34169210000255</v>
+        <v>13.42934260000038</v>
       </c>
     </row>
     <row r="5">
@@ -1178,10 +1282,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>80215041.95503481</v>
+        <v>30190010.59769762</v>
       </c>
       <c r="C5" t="n">
-        <v>12.24005570000008</v>
+        <v>12.76946969999699</v>
       </c>
     </row>
     <row r="6">
@@ -1189,10 +1293,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>80215041.95503481</v>
+        <v>30190010.59769762</v>
       </c>
       <c r="C6" t="n">
-        <v>15.11363210000127</v>
+        <v>12.75162090000231</v>
       </c>
     </row>
     <row r="7">
@@ -1200,10 +1304,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>80215041.95503481</v>
+        <v>30190010.59769762</v>
       </c>
       <c r="C7" t="n">
-        <v>14.44470189999993</v>
+        <v>10.87901299999794</v>
       </c>
     </row>
     <row r="8">
@@ -1211,10 +1315,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>80215041.95503481</v>
+        <v>42139026.10313972</v>
       </c>
       <c r="C8" t="n">
-        <v>12.75613980000344</v>
+        <v>12.72024860000238</v>
       </c>
     </row>
     <row r="9">
@@ -1222,10 +1326,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>80215041.95503481</v>
+        <v>42139026.10313972</v>
       </c>
       <c r="C9" t="n">
-        <v>11.71869770000194</v>
+        <v>11.06374729999516</v>
       </c>
     </row>
     <row r="10">
@@ -1233,10 +1337,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>80215041.95503481</v>
+        <v>42139026.10313972</v>
       </c>
       <c r="C10" t="n">
-        <v>14.81621520000044</v>
+        <v>14.04093550000107</v>
       </c>
     </row>
     <row r="11">
@@ -1244,10 +1348,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>80215041.95503481</v>
+        <v>42139026.10313972</v>
       </c>
       <c r="C11" t="n">
-        <v>12.12374350000027</v>
+        <v>13.94045129999722</v>
       </c>
     </row>
     <row r="12">
@@ -1255,10 +1359,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>80215041.95503481</v>
+        <v>42139026.10313972</v>
       </c>
       <c r="C12" t="n">
-        <v>13.30079770000157</v>
+        <v>11.12809320000088</v>
       </c>
     </row>
     <row r="13">
@@ -1266,10 +1370,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>80215041.95503481</v>
+        <v>42139026.10313972</v>
       </c>
       <c r="C13" t="n">
-        <v>9.830018000000564</v>
+        <v>13.88719110000238</v>
       </c>
     </row>
     <row r="14">
@@ -1277,10 +1381,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>80215041.95503481</v>
+        <v>42139026.10313972</v>
       </c>
       <c r="C14" t="n">
-        <v>15.64978859999974</v>
+        <v>11.81059729999834</v>
       </c>
     </row>
     <row r="15">
@@ -1288,10 +1392,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>80215041.95503481</v>
+        <v>61170857.59725153</v>
       </c>
       <c r="C15" t="n">
-        <v>10.35940760000085</v>
+        <v>13.46278440000606</v>
       </c>
     </row>
     <row r="16">
@@ -1299,10 +1403,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>80215041.95503481</v>
+        <v>61170857.59725153</v>
       </c>
       <c r="C16" t="n">
-        <v>12.80914029999985</v>
+        <v>13.21640990000014</v>
       </c>
     </row>
     <row r="17">
@@ -1310,10 +1414,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>86584661.52606127</v>
+        <v>61170857.59725153</v>
       </c>
       <c r="C17" t="n">
-        <v>14.39933500000188</v>
+        <v>15.53180900000007</v>
       </c>
     </row>
     <row r="18">
@@ -1321,10 +1425,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>86584661.52606127</v>
+        <v>61170857.59725153</v>
       </c>
       <c r="C18" t="n">
-        <v>15.1074105000007</v>
+        <v>11.78134839999984</v>
       </c>
     </row>
     <row r="19">
@@ -1332,10 +1436,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>86584661.52606127</v>
+        <v>67762141.22059186</v>
       </c>
       <c r="C19" t="n">
-        <v>15.56377470000007</v>
+        <v>13.71302239999932</v>
       </c>
     </row>
     <row r="20">
@@ -1343,10 +1447,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>94022632.97405255</v>
+        <v>72975469.68910632</v>
       </c>
       <c r="C20" t="n">
-        <v>15.3837790999969</v>
+        <v>14.91855139999825</v>
       </c>
     </row>
     <row r="21">
@@ -1354,10 +1458,340 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>94022632.97405255</v>
+        <v>76099191.12931634</v>
       </c>
       <c r="C21" t="n">
-        <v>15.38395650000166</v>
+        <v>15.20767559999513</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>76099191.12931634</v>
+      </c>
+      <c r="C22" t="n">
+        <v>12.69784589999472</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>76099191.12931634</v>
+      </c>
+      <c r="C23" t="n">
+        <v>15.08878149999509</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>76099191.12931634</v>
+      </c>
+      <c r="C24" t="n">
+        <v>10.73656749999645</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>76099191.12931634</v>
+      </c>
+      <c r="C25" t="n">
+        <v>14.95025579999492</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>76099191.12931634</v>
+      </c>
+      <c r="C26" t="n">
+        <v>14.27438190000248</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>76099191.12931634</v>
+      </c>
+      <c r="C27" t="n">
+        <v>8.738438299995323</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>76099191.12931634</v>
+      </c>
+      <c r="C28" t="n">
+        <v>14.16246789999423</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>78239642.08762258</v>
+      </c>
+      <c r="C29" t="n">
+        <v>14.19523599999957</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C30" t="n">
+        <v>15.09312120000686</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C31" t="n">
+        <v>12.92126049999933</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C32" t="n">
+        <v>13.13764829999855</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C33" t="n">
+        <v>15.80850199999986</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C34" t="n">
+        <v>14.49176090000401</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C35" t="n">
+        <v>10.24435770000127</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C36" t="n">
+        <v>13.02038309999625</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C37" t="n">
+        <v>15.30675199999678</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C38" t="n">
+        <v>15.21664050000254</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C39" t="n">
+        <v>14.59812149999925</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C40" t="n">
+        <v>13.41096510000352</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C41" t="n">
+        <v>12.3098691999985</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C42" t="n">
+        <v>13.65886740000133</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C43" t="n">
+        <v>11.26214009999967</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C44" t="n">
+        <v>10.93332019999798</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>78241502.26534167</v>
+      </c>
+      <c r="C45" t="n">
+        <v>12.81223850000242</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>79498938.60691604</v>
+      </c>
+      <c r="C46" t="n">
+        <v>14.79515159999573</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>79498938.60691604</v>
+      </c>
+      <c r="C47" t="n">
+        <v>15.45224430000235</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>79619862.0486231</v>
+      </c>
+      <c r="C48" t="n">
+        <v>15.30167459999939</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>79619862.0486231</v>
+      </c>
+      <c r="C49" t="n">
+        <v>11.69523109999864</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="n">
+        <v>79619862.0486231</v>
+      </c>
+      <c r="C50" t="n">
+        <v>12.6392418999967</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="n">
+        <v>80036495.78333437</v>
+      </c>
+      <c r="C51" t="n">
+        <v>12.03271189999941</v>
       </c>
     </row>
   </sheetData>

</xml_diff>